<commit_message>
Pushed changes for saas merged and alloction feature upto 4 April 24
</commit_message>
<xml_diff>
--- a/src/main/resources/AmendmentRequest_Field_Values.xlsx
+++ b/src/main/resources/AmendmentRequest_Field_Values.xlsx
@@ -1,45 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25330"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26529"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\product_automation\govgrants-product-automation\src\main\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\rei proj\Product_Auto_Clone\govgrants-product-automation\src\main\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59D6A6BC-3D67-4B6A-A9BB-0A71E8239ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98AA166-91E0-4F58-92C0-14DCADB4A3D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="135" yWindow="90" windowWidth="20370" windowHeight="10920" firstSheet="8" activeTab="9" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="7" activeTab="9" xr2:uid="{371138BB-CE66-4BB7-8C3C-9638AA0A141A}"/>
   </bookViews>
   <sheets>
     <sheet name="ScopeOfWork_Creation" sheetId="1" r:id="rId1"/>
     <sheet name="Scope&amp;BudgetPeriod_Creation" sheetId="25" r:id="rId2"/>
-    <sheet name="Subrecipient_SOW_creation" sheetId="17" r:id="rId3"/>
-    <sheet name="Budget_Redirection" sheetId="15" r:id="rId4"/>
-    <sheet name="Subrecipient_BRedirection" sheetId="21" r:id="rId5"/>
-    <sheet name="Subrecipient_KPC" sheetId="22" r:id="rId6"/>
-    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId7"/>
-    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId8"/>
-    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId9"/>
-    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId10"/>
-    <sheet name="Subrecipient_BPCSOW_Creation" sheetId="26" r:id="rId11"/>
-    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId12"/>
-    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId13"/>
-    <sheet name="SubRecipientCF_Creation" sheetId="23" r:id="rId14"/>
-    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId15"/>
-    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId16"/>
-    <sheet name="GrantCreation" sheetId="6" r:id="rId17"/>
-    <sheet name="GrantEdition" sheetId="7" r:id="rId18"/>
-    <sheet name="Edition_Standalone" sheetId="8" r:id="rId19"/>
-    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId20"/>
-    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId21"/>
-    <sheet name="Periodic Renewal" sheetId="12" r:id="rId22"/>
-    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId23"/>
-    <sheet name="Periodic Renewal Edition1" sheetId="28" r:id="rId24"/>
-    <sheet name="Funding_Terms_creation" sheetId="24" r:id="rId25"/>
-    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId26"/>
-    <sheet name="AllAmendment_Creation" sheetId="27" r:id="rId27"/>
+    <sheet name="BPC_SOW_FC_Creation" sheetId="30" r:id="rId3"/>
+    <sheet name="Subrecipient_SOW_creation" sheetId="17" r:id="rId4"/>
+    <sheet name="Budget_Redirection" sheetId="15" r:id="rId5"/>
+    <sheet name="Subrecipient_BRedirection" sheetId="21" r:id="rId6"/>
+    <sheet name="Subrecipient_BRedirec_Carry_Err" sheetId="29" r:id="rId7"/>
+    <sheet name="Subrecipient_KPC" sheetId="22" r:id="rId8"/>
+    <sheet name="ScopeOfWork_Edition" sheetId="2" r:id="rId9"/>
+    <sheet name="Subrecipient_SOW_Edition" sheetId="18" r:id="rId10"/>
+    <sheet name="BudgetPeriodChange_Creation" sheetId="3" r:id="rId11"/>
+    <sheet name="SubRecipientBPC_Creation" sheetId="19" r:id="rId12"/>
+    <sheet name="Subrecipient_BPCSOW_Creation" sheetId="26" r:id="rId13"/>
+    <sheet name="Sub_BR_KPC_SOW_creation" sheetId="31" r:id="rId14"/>
+    <sheet name="BudgetPeriodChange_Edition" sheetId="4" r:id="rId15"/>
+    <sheet name="SubRecipientBPC_Edition" sheetId="20" r:id="rId16"/>
+    <sheet name="SubRecipientCF_Creation" sheetId="23" r:id="rId17"/>
+    <sheet name="PaymentRequestEdition" sheetId="11" r:id="rId18"/>
+    <sheet name="FundingChange_Creation" sheetId="5" r:id="rId19"/>
+    <sheet name="GrantCreation" sheetId="6" r:id="rId20"/>
+    <sheet name="GrantEdition" sheetId="7" r:id="rId21"/>
+    <sheet name="Edition_Standalone" sheetId="8" r:id="rId22"/>
+    <sheet name="Payment Request Schedule" sheetId="9" r:id="rId23"/>
+    <sheet name="Progress Report Schedule" sheetId="10" r:id="rId24"/>
+    <sheet name="Periodic Renewal" sheetId="12" r:id="rId25"/>
+    <sheet name="Periodic Renewal Edition" sheetId="13" r:id="rId26"/>
+    <sheet name="Periodic Renewal Edition1" sheetId="28" r:id="rId27"/>
+    <sheet name="Funding_Terms_creation" sheetId="24" r:id="rId28"/>
+    <sheet name="TermsAndConditions_Creation" sheetId="14" r:id="rId29"/>
+    <sheet name="AllAmendment_Creation" sheetId="27" r:id="rId30"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="97">
   <si>
     <t>Sub Tab</t>
   </si>
@@ -129,9 +132,6 @@
     <t>Congressionaldistrict__c</t>
   </si>
   <si>
-    <t>1st District</t>
-  </si>
-  <si>
     <t>Budget Period Change</t>
   </si>
   <si>
@@ -327,12 +327,6 @@
     <t>fieldCounty__c</t>
   </si>
   <si>
-    <t>Automation Country</t>
-  </si>
-  <si>
-    <t>KA</t>
-  </si>
-  <si>
     <t>fieldState__c</t>
   </si>
   <si>
@@ -355,6 +349,12 @@
   </si>
   <si>
     <t>fieldAddressline2__c</t>
+  </si>
+  <si>
+    <t>fieldRevisedCommitment__c</t>
+  </si>
+  <si>
+    <t>USA</t>
   </si>
 </sst>
 </file>
@@ -782,7 +782,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -817,6 +817,189 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2B8548-7B25-4129-9EB7-BF1BA0DF00C4}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.42578125" customWidth="1"/>
+    <col min="3" max="3" width="44" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="C3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8">
+        <v>12345</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="C9">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
+  <dimension ref="A1:C4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25797962-2CD8-4222-8F0C-F2737F68CB74}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -841,10 +1024,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -852,7 +1035,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -863,7 +1046,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -875,7 +1058,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6EBA5DFF-498D-4D83-B948-A4DE3D93557A}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -900,10 +1083,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -911,7 +1094,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>
@@ -922,7 +1105,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -933,7 +1116,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
         <v>6</v>
@@ -944,7 +1127,86 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7391CE8D-3E64-4DF2-B815-01A045EEFFCE}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="C4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46AF2254-AE3B-4E5C-85F3-E6BD713DEDBA}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -969,7 +1231,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -980,10 +1242,10 @@
         <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -992,7 +1254,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F116B932-6CC5-49E6-907B-B1FB48B4CADD}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1018,7 +1280,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C2">
         <v>70</v>
@@ -1029,10 +1291,10 @@
         <v>12</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>
@@ -1040,7 +1302,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AFB9B001-FDE9-4CB7-8749-6B43410AD625}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1065,10 +1327,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1076,7 +1338,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -1087,7 +1349,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1098,7 +1360,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5E7F2A7-80D1-499C-A4FA-A74EFAC3E1B6}">
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1120,24 +1382,24 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" t="s">
         <v>68</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>69</v>
-      </c>
-      <c r="C2" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C3" t="s">
         <v>71</v>
-      </c>
-      <c r="C3" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1145,7 +1407,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F7F1F928-5062-4480-A5CB-C00A65CDBE7D}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1170,10 +1432,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1201,312 +1463,6 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5">
-        <v>3650</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" t="s">
-        <v>38</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C3" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-      <c r="B8" t="s">
-        <v>47</v>
-      </c>
-      <c r="C8" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>3</v>
-      </c>
-      <c r="B9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>3</v>
-      </c>
-      <c r="B10" t="s">
-        <v>49</v>
-      </c>
-      <c r="C10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>3</v>
-      </c>
-      <c r="B11" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>3</v>
-      </c>
-      <c r="B12" t="s">
-        <v>51</v>
-      </c>
-      <c r="C12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C2" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3">
-        <v>3650</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -1535,7 +1491,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -1546,10 +1502,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1580,6 +1536,312 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51772752-268C-420F-8F6C-3EB44DC586C7}">
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="38.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5">
+        <v>3650</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D1BAA82-C6A0-43F4-ACD7-0F51FAC17BDE}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="30.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>38</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>3</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>3</v>
+      </c>
+      <c r="B9" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B11" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>3</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
+      </c>
+      <c r="C12" t="s">
+        <v>39</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B98C2E6-0C38-44BD-BCCA-D74A75F16055}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="25" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C3">
+        <v>3650</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36CE4AB1-D2A4-48AD-BE1D-510D3EC12A32}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1604,10 +1866,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" t="s">
         <v>56</v>
-      </c>
-      <c r="C2" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1615,10 +1877,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1626,10 +1888,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1637,10 +1899,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1648,7 +1910,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1659,7 +1921,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -1670,7 +1932,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6AF52C3-BB99-4CC4-A56A-57677D233764}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1695,10 +1957,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1706,10 +1968,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" t="s">
         <v>58</v>
-      </c>
-      <c r="C3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1717,10 +1979,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C4" t="s">
         <v>60</v>
-      </c>
-      <c r="C4" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1728,10 +1990,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1739,7 +2001,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1750,7 +2012,7 @@
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C7">
         <v>3650</v>
@@ -1761,7 +2023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAF2024B-3855-4F21-818F-72BDEF018EB6}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1786,10 +2048,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1797,7 +2059,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -1808,7 +2070,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -1819,7 +2081,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D6731B0-0A3A-4C99-9219-CD51FBCA919D}">
   <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1844,7 +2106,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C2" s="5">
         <v>4017</v>
@@ -1855,7 +2117,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>1000</v>
@@ -1866,10 +2128,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1877,10 +2139,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1888,10 +2150,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1899,14 +2161,22 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="B8" s="7"/>
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8">
+        <v>2000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1914,9 +2184,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{553CC38A-2DBF-46D2-8E76-C45CC7EF93DF}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" bestFit="1" customWidth="1"/>
@@ -1939,7 +2209,7 @@
         <v>12</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C2" s="5">
         <v>6017</v>
@@ -1950,7 +2220,7 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C3">
         <v>1000</v>
@@ -1961,10 +2231,10 @@
         <v>12</v>
       </c>
       <c r="B4" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1972,10 +2242,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1983,10 +2253,10 @@
         <v>12</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C6" t="s">
-        <v>89</v>
+        <v>80</v>
+      </c>
+      <c r="C6">
+        <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1994,10 +2264,21 @@
         <v>12</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8">
+        <v>3000</v>
       </c>
     </row>
   </sheetData>
@@ -2005,7 +2286,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet28.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62770C67-3364-43CF-8FC9-172E7743FC1C}">
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2030,10 +2311,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2041,10 +2322,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2074,7 +2355,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet29.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C01F7F05-2D11-4E6A-A090-87D63AD5B8AF}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2099,10 +2380,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2132,7 +2413,87 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet27.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD4347D0-7C7B-4991-B39A-D56700E62FF3}">
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DFDBA76-585A-4956-AF61-28921A0073B1}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2157,7 +2518,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -2168,10 +2529,10 @@
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -2179,10 +2540,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -2190,10 +2551,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2223,7 +2584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE5594E6-CDC4-4068-99A2-0F1E0C84230B}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2249,7 +2610,7 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
@@ -2260,7 +2621,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2271,7 +2632,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2283,7 +2644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CED252CC-9A41-43A8-97A3-527BD171EFF4}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2309,10 +2670,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2343,7 +2704,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1C7C3E9-7A91-479E-8DB7-C5289494DF22}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2368,10 +2729,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2379,7 +2740,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2390,7 +2751,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2402,7 +2763,76 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FA7DC5-C4A1-4E9C-B02D-9945A615B758}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>76</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F956442-5D32-41A9-9373-4CEFD36ACD4B}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2427,10 +2857,10 @@
         <v>3</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -2438,7 +2868,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C3" t="s">
         <v>6</v>
@@ -2449,7 +2879,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
         <v>6</v>
@@ -2460,7 +2890,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF3C3D45-7E71-472A-AB14-3D5373D782BA}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2551,11 +2981,11 @@
       <c r="A8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
-        <v>86</v>
+      <c r="B8" s="7" t="s">
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -2576,8 +3006,8 @@
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" t="s">
-        <v>22</v>
+      <c r="C10">
+        <v>123</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -2585,193 +3015,10 @@
         <v>12</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C11" t="s">
         <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1B2B8548-7B25-4129-9EB7-BF1BA0DF00C4}">
-  <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.42578125" customWidth="1"/>
-    <col min="3" max="3" width="44" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="7" t="s">
-        <v>79</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>94</v>
-      </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="C7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>20</v>
-      </c>
-      <c r="C8">
-        <v>12345</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="C9" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="C10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF0DD9D3-0F99-4CAD-B5E8-028A0FF50760}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="2" max="2" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>